<commit_message>
2035 RES constraint's interpolation rule set to 5
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962887BF-7A4A-4A86-AAA9-B65865038A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AEB3EB9-1F7A-473A-BBD9-19FAE80E54E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -510,7 +510,7 @@
         <v>0</v>
       </c>
       <c r="M6">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="N6" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Adding constraint to bio energy
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BEF9F41-8248-46CC-AA7E-F2C9CBE071CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02B49C3B-E597-40BD-8C96-A822FEA1D341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -99,6 +99,24 @@
   </si>
   <si>
     <t>~UC_Sets: R_E: AllRegions</t>
+  </si>
+  <si>
+    <t>UC_CAP</t>
+  </si>
+  <si>
+    <t>UC_RHSRT</t>
+  </si>
+  <si>
+    <t>UC_RHSRT~0</t>
+  </si>
+  <si>
+    <t>ep_bioenergy*,bioen*</t>
+  </si>
+  <si>
+    <t>~UC_T: UC_CAP~UP</t>
+  </si>
+  <si>
+    <t>UCE_max_bio_capacity</t>
   </si>
 </sst>
 </file>
@@ -433,23 +451,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:N7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:N11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="31.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.26953125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
+    <row r="1" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
+    </row>
+    <row r="2" spans="2:14" x14ac:dyDescent="0.35">
       <c r="E2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.35">
       <c r="J4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B5" s="2" t="s">
         <v>2</v>
       </c>
@@ -490,7 +518,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>15</v>
       </c>
@@ -522,9 +550,48 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Adding constraint to bio energy, attempt 2
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02B49C3B-E597-40BD-8C96-A822FEA1D341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5805EEF-9C67-43F2-BE1E-0F6985060CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -104,19 +104,19 @@
     <t>UC_CAP</t>
   </si>
   <si>
-    <t>UC_RHSRT</t>
-  </si>
-  <si>
-    <t>UC_RHSRT~0</t>
-  </si>
-  <si>
     <t>ep_bioenergy*,bioen*</t>
   </si>
   <si>
-    <t>~UC_T: UC_CAP~UP</t>
-  </si>
-  <si>
     <t>UCE_max_bio_capacity</t>
+  </si>
+  <si>
+    <t>UP</t>
+  </si>
+  <si>
+    <t>~UC_T:UC_RHSRTS</t>
+  </si>
+  <si>
+    <t>Maximum capacity allowed of bioenergy powerplants</t>
   </si>
 </sst>
 </file>
@@ -166,11 +166,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -456,9 +457,11 @@
   <cols>
     <col min="2" max="2" width="31.90625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.26953125" customWidth="1"/>
     <col min="10" max="10" width="18.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -555,7 +558,7 @@
       <c r="M7" s="3"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B9" t="s">
+      <c r="D9" t="s">
         <v>25</v>
       </c>
     </row>
@@ -564,36 +567,43 @@
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" t="s">
         <v>21</v>
       </c>
-      <c r="E10" t="s">
-        <v>22</v>
-      </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>11</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" t="s">
         <v>24</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>1</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
       </c>
       <c r="F11">
         <v>3</v>
       </c>
+      <c r="G11" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Setting capacity sum of bioenergy powerplants max to 1 GW
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F3BE7A-C339-4234-821C-1F7E9D54E7A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F75944-18B3-41D5-97F2-00B00E4A309F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -598,7 +598,7 @@
         <v>1</v>
       </c>
       <c r="F11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G11" t="s">
         <v>25</v>

</xml_diff>

<commit_message>
attempt 2: Setting capacity sum of bioenergy powerplants max to 1 GW
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F75944-18B3-41D5-97F2-00B00E4A309F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C702FB81-A10C-4A8E-9C55-ECC5917AA665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -110,9 +110,6 @@
     <t>UP</t>
   </si>
   <si>
-    <t>~UC_T:UC_RHSRTS</t>
-  </si>
-  <si>
     <t>Maximum capacity allowed of bioenergy powerplants</t>
   </si>
   <si>
@@ -120,6 +117,24 @@
   </si>
   <si>
     <t>bioenergy</t>
+  </si>
+  <si>
+    <t>~UC_T: 2050</t>
+  </si>
+  <si>
+    <t>pset_co</t>
+  </si>
+  <si>
+    <t>UC_ACT</t>
+  </si>
+  <si>
+    <t>UC_RHSRT</t>
+  </si>
+  <si>
+    <t>UC_RHSRT~0</t>
+  </si>
+  <si>
+    <t>UC_T:UC_RHSRTS</t>
   </si>
 </sst>
 </file>
@@ -454,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:N11"/>
+  <dimension ref="B1:N13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="31.90625" bestFit="1" customWidth="1"/>
@@ -464,6 +479,7 @@
     <col min="6" max="6" width="13.6328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5.26953125" customWidth="1"/>
+    <col min="9" max="9" width="9.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -559,49 +575,100 @@
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
     </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+    </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>25</v>
+      </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9">
+        <v>2022</v>
+      </c>
+      <c r="H9">
+        <v>2050</v>
+      </c>
+      <c r="I9" t="s">
+        <v>30</v>
+      </c>
+      <c r="J9" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B13" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" t="s">
         <v>26</v>
       </c>
-      <c r="D10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="D13" t="s">
         <v>23</v>
       </c>
-      <c r="E11">
+      <c r="E13">
         <v>1</v>
       </c>
-      <c r="F11">
+      <c r="F13">
         <v>1</v>
       </c>
-      <c r="G11" t="s">
-        <v>25</v>
+      <c r="G13" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
attempt 3: Setting capacity sum of bioenergy powerplants max to 1 GW
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C702FB81-A10C-4A8E-9C55-ECC5917AA665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED506256-5EC6-40A9-B999-88E7FC205E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -119,9 +119,6 @@
     <t>bioenergy</t>
   </si>
   <si>
-    <t>~UC_T: 2050</t>
-  </si>
-  <si>
     <t>pset_co</t>
   </si>
   <si>
@@ -134,7 +131,13 @@
     <t>UC_RHSRT~0</t>
   </si>
   <si>
-    <t>UC_T:UC_RHSRTS</t>
+    <t>*UC_T: 2050</t>
+  </si>
+  <si>
+    <t>~UC_Sets: T_E:</t>
+  </si>
+  <si>
+    <t>~UC_T:UC_RHSRTS</t>
   </si>
 </sst>
 </file>
@@ -469,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:N13"/>
+  <dimension ref="B1:N35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="31.90625" bestFit="1" customWidth="1"/>
@@ -477,8 +480,7 @@
     <col min="4" max="4" width="16.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.26953125" customWidth="1"/>
+    <col min="7" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.26953125" bestFit="1" customWidth="1"/>
   </cols>
@@ -575,99 +577,122 @@
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
     </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B9" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9">
-        <v>2022</v>
-      </c>
-      <c r="H9">
-        <v>2050</v>
-      </c>
-      <c r="I9" t="s">
-        <v>30</v>
-      </c>
-      <c r="J9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="I10">
-        <v>1</v>
-      </c>
-      <c r="J10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="D11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
-        <v>2</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="E14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" t="s">
+        <v>30</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
         <v>22</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C16" t="s">
         <v>26</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D16">
+        <v>2022</v>
+      </c>
+      <c r="E16" t="s">
         <v>23</v>
       </c>
-      <c r="E13">
+      <c r="F16">
         <v>1</v>
       </c>
-      <c r="F13">
+      <c r="G16">
         <v>1</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H16">
+        <v>15</v>
+      </c>
+      <c r="I16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B33" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B34" t="s">
+        <v>2</v>
+      </c>
+      <c r="C34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D34" t="s">
+        <v>27</v>
+      </c>
+      <c r="E34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F34" t="s">
+        <v>21</v>
+      </c>
+      <c r="G34">
+        <v>2022</v>
+      </c>
+      <c r="H34">
+        <v>2050</v>
+      </c>
+      <c r="I34" t="s">
+        <v>29</v>
+      </c>
+      <c r="J34" t="s">
+        <v>30</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B35" t="s">
+        <v>22</v>
+      </c>
+      <c r="C35" t="s">
+        <v>26</v>
+      </c>
+      <c r="F35">
+        <v>1</v>
+      </c>
+      <c r="I35">
+        <v>1</v>
+      </c>
+      <c r="J35">
+        <v>3</v>
+      </c>
+      <c r="K35" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
attempt 4: Setting capacity sum of bioenergy powerplants max to 1 GW
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED506256-5EC6-40A9-B999-88E7FC205E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBFA924-7399-4273-B613-2BA781BA6663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -137,7 +137,7 @@
     <t>~UC_Sets: T_E:</t>
   </si>
   <si>
-    <t>~UC_T:UC_RHSRTS</t>
+    <t>~UC_T:UC_RHSRT</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
attempt 5: Setting capacity sum of bioenergy powerplants max to 1 GW
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBFA924-7399-4273-B613-2BA781BA6663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5353B45A-49E3-4812-A5B4-7CAACC14913F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -577,6 +577,11 @@
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
     </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+    </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>32</v>
@@ -637,6 +642,20 @@
       </c>
       <c r="I16" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="3:6" x14ac:dyDescent="0.35">
+      <c r="C17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17">
+        <v>2050</v>
+      </c>
+      <c r="E17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
attempt 6: Setting capacity sum of bioenergy powerplants max to 1 GW
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5353B45A-49E3-4812-A5B4-7CAACC14913F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDF18AB0-7686-45C5-9FAE-604BA46F7C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -483,6 +483,7 @@
     <col min="7" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:14" x14ac:dyDescent="0.35">
@@ -612,7 +613,7 @@
         <v>11</v>
       </c>
       <c r="H15" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
attempt 7: Setting capacity sum of bioenergy powerplants max to 1 GW
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDF18AB0-7686-45C5-9FAE-604BA46F7C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E89BA6BF-1F61-47E2-8514-372418AB6D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="35">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -138,6 +138,9 @@
   </si>
   <si>
     <t>~UC_T:UC_RHSRT</t>
+  </si>
+  <si>
+    <t>Bio Power</t>
   </si>
 </sst>
 </file>
@@ -480,7 +483,8 @@
     <col min="4" max="4" width="16.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.54296875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.26953125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.6328125" bestFit="1" customWidth="1"/>
@@ -597,25 +601,28 @@
       <c r="B15" t="s">
         <v>2</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>9</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>21</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>11</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>13</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -624,38 +631,41 @@
         <v>22</v>
       </c>
       <c r="C16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" t="s">
         <v>26</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>2022</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>23</v>
-      </c>
-      <c r="F16">
-        <v>1</v>
       </c>
       <c r="G16">
         <v>1</v>
       </c>
       <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
         <v>15</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.35">
-      <c r="C17" t="s">
+    <row r="17" spans="4:7" x14ac:dyDescent="0.35">
+      <c r="D17" t="s">
         <v>26</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>2050</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>23</v>
       </c>
-      <c r="F17">
+      <c r="G17">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
attempt 8: Setting capacity sum of bioenergy powerplants max to 1 GW
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E89BA6BF-1F61-47E2-8514-372418AB6D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0EC6E30-22B4-4DAC-BC92-69DFB8E0FFDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -484,9 +484,9 @@
     <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="12.54296875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -620,7 +620,7 @@
         <v>11</v>
       </c>
       <c r="I15" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
attempt 9: Setting capacity sum of bioenergy powerplants max to 1 GW
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0EC6E30-22B4-4DAC-BC92-69DFB8E0FFDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E95CFFC-56AD-42E4-8C70-BA702FA0519C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="35">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -633,9 +633,6 @@
       <c r="C16" t="s">
         <v>34</v>
       </c>
-      <c r="D16" t="s">
-        <v>26</v>
-      </c>
       <c r="E16">
         <v>2022</v>
       </c>
@@ -655,9 +652,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="4:7" x14ac:dyDescent="0.35">
-      <c r="D17" t="s">
-        <v>26</v>
+    <row r="17" spans="3:7" x14ac:dyDescent="0.35">
+      <c r="C17" t="s">
+        <v>34</v>
       </c>
       <c r="E17">
         <v>2050</v>

</xml_diff>

<commit_message>
attempt 10: Setting capacity sum of bioenergy powerplants max to 1 GW
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E95CFFC-56AD-42E4-8C70-BA702FA0519C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D9FBA7-0A33-4CB2-88CC-E51BA29FC681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="35">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -633,6 +633,9 @@
       <c r="C16" t="s">
         <v>34</v>
       </c>
+      <c r="D16" t="s">
+        <v>26</v>
+      </c>
       <c r="E16">
         <v>2022</v>
       </c>
@@ -643,7 +646,7 @@
         <v>1</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="I16">
         <v>15</v>
@@ -655,6 +658,9 @@
     <row r="17" spans="3:7" x14ac:dyDescent="0.35">
       <c r="C17" t="s">
         <v>34</v>
+      </c>
+      <c r="D17" t="s">
+        <v>26</v>
       </c>
       <c r="E17">
         <v>2050</v>

</xml_diff>

<commit_message>
Attempt 4: Fix constraint of renewable production
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D9FBA7-0A33-4CB2-88CC-E51BA29FC681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{078023FE-C1E2-4B3B-B50B-23629F1275C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -83,9 +83,6 @@
     <t>UC_Desc</t>
   </si>
   <si>
-    <t>UC_min_renew_20235</t>
-  </si>
-  <si>
     <t>PP_RENEW</t>
   </si>
   <si>
@@ -140,7 +137,7 @@
     <t>~UC_T:UC_RHSRT</t>
   </si>
   <si>
-    <t>Bio Power</t>
+    <t>UC_min_renew_2035</t>
   </si>
 </sst>
 </file>
@@ -497,7 +494,7 @@
     </row>
     <row r="2" spans="2:14" x14ac:dyDescent="0.35">
       <c r="E2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.35">
@@ -548,19 +545,19 @@
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" t="s">
+      <c r="G6" t="s">
         <v>16</v>
-      </c>
-      <c r="G6" t="s">
-        <v>17</v>
       </c>
       <c r="H6">
         <v>2035</v>
       </c>
       <c r="I6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -575,7 +572,7 @@
         <v>5</v>
       </c>
       <c r="N6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.35">
@@ -584,97 +581,88 @@
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D14" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="E14" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>2</v>
       </c>
-      <c r="C15" t="s">
-        <v>3</v>
+      <c r="C15" s="2" t="s">
+        <v>24</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E15" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="E15" t="s">
+        <v>9</v>
+      </c>
       <c r="F15" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="G15" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="H15" t="s">
-        <v>11</v>
-      </c>
-      <c r="I15" t="s">
-        <v>30</v>
-      </c>
-      <c r="J15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16">
+        <v>2022</v>
+      </c>
+      <c r="E16" t="s">
         <v>22</v>
       </c>
-      <c r="C16" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16" t="s">
-        <v>26</v>
-      </c>
-      <c r="E16">
-        <v>2022</v>
-      </c>
-      <c r="F16" t="s">
-        <v>23</v>
+      <c r="F16">
+        <v>1</v>
       </c>
       <c r="G16">
         <v>1</v>
       </c>
       <c r="H16">
-        <v>0.01</v>
-      </c>
-      <c r="I16">
         <v>15</v>
       </c>
-      <c r="J16" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.35">
+      <c r="I16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="3:6" x14ac:dyDescent="0.35">
       <c r="C17" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" t="s">
-        <v>26</v>
-      </c>
-      <c r="E17">
+        <v>25</v>
+      </c>
+      <c r="D17">
         <v>2050</v>
       </c>
-      <c r="F17" t="s">
-        <v>23</v>
-      </c>
-      <c r="G17">
+      <c r="E17" t="s">
+        <v>22</v>
+      </c>
+      <c r="F17">
         <v>1</v>
       </c>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.35">
@@ -682,16 +670,16 @@
         <v>2</v>
       </c>
       <c r="C34" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D34" t="s">
+        <v>26</v>
+      </c>
+      <c r="E34" t="s">
         <v>27</v>
       </c>
-      <c r="E34" t="s">
-        <v>28</v>
-      </c>
       <c r="F34" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G34">
         <v>2022</v>
@@ -700,10 +688,10 @@
         <v>2050</v>
       </c>
       <c r="I34" t="s">
+        <v>28</v>
+      </c>
+      <c r="J34" t="s">
         <v>29</v>
-      </c>
-      <c r="J34" t="s">
-        <v>30</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>14</v>
@@ -711,10 +699,10 @@
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B35" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C35" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F35">
         <v>1</v>
@@ -726,7 +714,7 @@
         <v>3</v>
       </c>
       <c r="K35" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Attemps 2: Testing solid power plants constraint
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B2480B4-6C8D-4FB5-99E5-4B33B27961C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDF8CA7-5065-4CC7-8003-FD85B32C68F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="37">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -584,35 +584,6 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
-        <v>34</v>
-      </c>
-      <c r="G7" t="s">
-        <v>35</v>
-      </c>
-      <c r="H7">
-        <v>2035</v>
-      </c>
-      <c r="I7" t="s">
-        <v>17</v>
-      </c>
-      <c r="J7">
-        <v>1</v>
-      </c>
-      <c r="K7">
-        <v>-20</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>5</v>
-      </c>
-      <c r="N7" t="s">
-        <v>36</v>
-      </c>
-    </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>19</v>
@@ -624,7 +595,7 @@
       </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>32</v>
       </c>
     </row>
@@ -636,21 +607,24 @@
         <v>24</v>
       </c>
       <c r="D15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>9</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>20</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>11</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>29</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -661,37 +635,63 @@
       <c r="C16" t="s">
         <v>25</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>2022</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>22</v>
-      </c>
-      <c r="F16">
-        <v>1</v>
       </c>
       <c r="G16">
         <v>1</v>
       </c>
       <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
         <v>15</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C17" t="s">
         <v>25</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>2050</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>22</v>
       </c>
-      <c r="F17">
+      <c r="G17">
         <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18">
+        <v>2035</v>
+      </c>
+      <c r="F18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>1.2</v>
+      </c>
+      <c r="I18">
+        <v>15</v>
+      </c>
+      <c r="J18" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Attemps 4: Testing solid power plants constraint
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BDB05D-E788-4F5E-AEB7-82FE3B7EED6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D1D9D3-C6E8-44F5-885F-2E3DB1EEF085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -654,7 +654,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
       <c r="D17" t="s">
         <v>25</v>
       </c>
@@ -668,29 +668,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>34</v>
       </c>
       <c r="C18" t="s">
         <v>36</v>
       </c>
-      <c r="F18">
+      <c r="E18">
         <v>2035</v>
       </c>
-      <c r="G18" t="s">
+      <c r="F18" t="s">
         <v>17</v>
       </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
       <c r="H18">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="I18">
-        <v>1.2</v>
-      </c>
-      <c r="J18">
         <v>15</v>
       </c>
-      <c r="K18" t="s">
+      <c r="J18" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Commenting out solid fuel constraint
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25C15AF4-CB98-42EE-821F-11A06B65E5AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32156E68-7416-4602-BDAD-1532F5FDCDF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -668,29 +668,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B18" t="s">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B20" t="s">
         <v>34</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C20" t="s">
         <v>36</v>
       </c>
-      <c r="E18">
+      <c r="E20">
         <v>2035</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F20" t="s">
         <v>17</v>
       </c>
-      <c r="G18">
+      <c r="G20">
         <v>1</v>
       </c>
-      <c r="H18">
+      <c r="H20">
         <v>2.1</v>
       </c>
-      <c r="I18">
+      <c r="I20">
         <v>15</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J20" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Attempt 6: Testing solid power plants constraint
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32156E68-7416-4602-BDAD-1532F5FDCDF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F36AFD2-663A-4394-9AF4-3EAE12DCF13E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -668,29 +668,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B20" t="s">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B18" t="s">
         <v>34</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C18" t="s">
         <v>36</v>
       </c>
-      <c r="E20">
+      <c r="E18">
         <v>2035</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F18" t="s">
         <v>17</v>
       </c>
-      <c r="G20">
+      <c r="G18">
         <v>1</v>
       </c>
-      <c r="H20">
+      <c r="H18">
         <v>2.1</v>
       </c>
-      <c r="I20">
-        <v>15</v>
-      </c>
-      <c r="J20" t="s">
+      <c r="I18">
+        <v>5</v>
+      </c>
+      <c r="J18" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Attempt 7: Testing solid power plants constraint
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F36AFD2-663A-4394-9AF4-3EAE12DCF13E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{857D286A-458B-4E67-80C0-371BA3F84826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="37">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -676,7 +676,7 @@
         <v>36</v>
       </c>
       <c r="E18">
-        <v>2035</v>
+        <v>2030</v>
       </c>
       <c r="F18" t="s">
         <v>17</v>
@@ -685,13 +685,30 @@
         <v>1</v>
       </c>
       <c r="H18">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="I18">
         <v>5</v>
       </c>
       <c r="J18" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="C19" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19">
+        <v>2035</v>
+      </c>
+      <c r="F19" t="s">
+        <v>17</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>2.1</v>
       </c>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Adding range of renewable by 2035 (75%-85%)
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{857D286A-458B-4E67-80C0-371BA3F84826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01222AC1-BC21-4FA7-A392-4E568BAA9194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="37">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -572,7 +572,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="3">
-        <v>-0.65</v>
+        <v>-0.75</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -582,6 +582,29 @@
       </c>
       <c r="N6" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7">
+        <v>2035</v>
+      </c>
+      <c r="I7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7" s="3">
+        <v>-0.85</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
attempt 2: Adding range of renewable by 2035 (75%-85%)
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01222AC1-BC21-4FA7-A392-4E568BAA9194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64DCEDE9-7604-493C-A38B-3E8774DEC9AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -147,6 +147,12 @@
   </si>
   <si>
     <t>pp_controllable</t>
+  </si>
+  <si>
+    <t>UC_max_renew_2035</t>
+  </si>
+  <si>
+    <t>Maximum renewable power plants penetration</t>
   </si>
 </sst>
 </file>
@@ -585,6 +591,9 @@
       </c>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
       <c r="C7" t="s">
         <v>15</v>
       </c>
@@ -605,6 +614,12 @@
       </c>
       <c r="L7">
         <v>0</v>
+      </c>
+      <c r="M7">
+        <v>5</v>
+      </c>
+      <c r="N7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Removing ELC FOR CSet_CN from renewable constraints
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64DCEDE9-7604-493C-A38B-3E8774DEC9AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B051C93C-DC4A-4824-B421-B3DC1A506BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="38">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -84,9 +84,6 @@
   </si>
   <si>
     <t>PP_RENEW</t>
-  </si>
-  <si>
-    <t>ELC</t>
   </si>
   <si>
     <t>LO</t>
@@ -509,7 +506,7 @@
     </row>
     <row r="2" spans="2:14" x14ac:dyDescent="0.35">
       <c r="E2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.35">
@@ -560,19 +557,16 @@
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
         <v>15</v>
       </c>
-      <c r="G6" t="s">
-        <v>16</v>
-      </c>
       <c r="H6">
         <v>2035</v>
       </c>
       <c r="I6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -587,24 +581,21 @@
         <v>5</v>
       </c>
       <c r="N6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
         <v>15</v>
       </c>
-      <c r="G7" t="s">
-        <v>16</v>
-      </c>
       <c r="H7">
         <v>2035</v>
       </c>
       <c r="I7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -619,22 +610,22 @@
         <v>5</v>
       </c>
       <c r="N7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.35">
       <c r="E14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="2:14" x14ac:dyDescent="0.35">
@@ -645,7 +636,7 @@
         <v>3</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>8</v>
@@ -654,13 +645,13 @@
         <v>9</v>
       </c>
       <c r="G15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
       </c>
       <c r="I15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>14</v>
@@ -668,16 +659,16 @@
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E16">
         <v>2022</v>
       </c>
       <c r="F16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -689,18 +680,18 @@
         <v>15</v>
       </c>
       <c r="J16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.35">
       <c r="D17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E17">
         <v>2050</v>
       </c>
       <c r="F17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -708,16 +699,16 @@
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E18">
         <v>2030</v>
       </c>
       <c r="F18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G18">
         <v>1</v>
@@ -729,18 +720,18 @@
         <v>5</v>
       </c>
       <c r="J18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E19">
         <v>2035</v>
       </c>
       <c r="F19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G19">
         <v>1</v>
@@ -751,7 +742,7 @@
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.35">
@@ -759,16 +750,16 @@
         <v>2</v>
       </c>
       <c r="C34" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D34" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34" t="s">
         <v>26</v>
       </c>
-      <c r="E34" t="s">
-        <v>27</v>
-      </c>
       <c r="F34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G34">
         <v>2022</v>
@@ -777,10 +768,10 @@
         <v>2050</v>
       </c>
       <c r="I34" t="s">
+        <v>27</v>
+      </c>
+      <c r="J34" t="s">
         <v>28</v>
-      </c>
-      <c r="J34" t="s">
-        <v>29</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>14</v>
@@ -788,10 +779,10 @@
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F35">
         <v>1</v>
@@ -803,7 +794,7 @@
         <v>3</v>
       </c>
       <c r="K35" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding ELC back for CSet_CN from renewable constraints and removing PSet_CN == PP_RENEW
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B051C93C-DC4A-4824-B421-B3DC1A506BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A0E91B6-441D-480C-B2BA-6F190E5A849D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
     <t>UC_Desc</t>
   </si>
   <si>
-    <t>PP_RENEW</t>
+    <t>ELC</t>
   </si>
   <si>
     <t>LO</t>
@@ -559,7 +559,7 @@
       <c r="B6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" t="s">
+      <c r="G6" t="s">
         <v>15</v>
       </c>
       <c r="H6">
@@ -588,7 +588,7 @@
       <c r="B7" t="s">
         <v>36</v>
       </c>
-      <c r="C7" t="s">
+      <c r="G7" t="s">
         <v>15</v>
       </c>
       <c r="H7">

</xml_diff>

<commit_message>
Commenting out bioenergy constraints
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB7105A-A781-489D-B3D7-8C21B47ED04B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BA121B4-5044-4C48-8125-65B99D36848E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -668,85 +668,85 @@
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16">
+        <v>2030</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>2</v>
+      </c>
+      <c r="I16">
+        <v>5</v>
+      </c>
+      <c r="J16" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="C17" t="s">
+        <v>36</v>
+      </c>
+      <c r="E17">
+        <v>2035</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
         <v>21</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D22" t="s">
         <v>25</v>
       </c>
-      <c r="E16">
+      <c r="E22">
         <v>2022</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F22" t="s">
         <v>22</v>
       </c>
-      <c r="G16">
-        <v>1</v>
-      </c>
-      <c r="H16">
-        <v>1</v>
-      </c>
-      <c r="I16">
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+      <c r="I22">
         <v>15</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J22" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="D17" t="s">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="D23" t="s">
         <v>25</v>
       </c>
-      <c r="E17">
+      <c r="E23">
         <v>2050</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F23" t="s">
         <v>22</v>
       </c>
-      <c r="G17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B18" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" t="s">
-        <v>36</v>
-      </c>
-      <c r="E18">
-        <v>2030</v>
-      </c>
-      <c r="F18" t="s">
-        <v>17</v>
-      </c>
-      <c r="G18">
-        <v>1</v>
-      </c>
-      <c r="H18">
-        <v>2</v>
-      </c>
-      <c r="I18">
-        <v>5</v>
-      </c>
-      <c r="J18" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="C19" t="s">
-        <v>36</v>
-      </c>
-      <c r="E19">
-        <v>2035</v>
-      </c>
-      <c r="F19" t="s">
-        <v>17</v>
-      </c>
-      <c r="G19">
-        <v>1</v>
-      </c>
-      <c r="H19">
-        <v>2.1</v>
+      <c r="G23">
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Correcting of min max renewable constraints
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BA121B4-5044-4C48-8125-65B99D36848E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C7C6394-6BFE-410C-B140-A4F78371B0CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -513,7 +513,7 @@
       </c>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="J4" t="s">
+      <c r="I4" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adding missing oil power plants
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C7C6394-6BFE-410C-B140-A4F78371B0CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31A9C77-CC86-4B38-8BFC-972D16277EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Disabling battery storage related processes by setting their start time outside the horion (2100)
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31A9C77-CC86-4B38-8BFC-972D16277EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40442FEC-BF39-4188-88E8-7BB3F5B68F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,8 +35,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={00A4DA71-5044-48BD-9C8D-CB976CA816BD}</author>
+  </authors>
+  <commentList>
+    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{00A4DA71-5044-48BD-9C8D-CB976CA816BD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Disabling battery storage related technologies by setting their start time outside the monitored horizon</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="45">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -153,13 +171,31 @@
   </si>
   <si>
     <t>Maximum renewable power plants penetration</t>
+  </si>
+  <si>
+    <t>Disabled:</t>
+  </si>
+  <si>
+    <t>~TFM_INS</t>
+  </si>
+  <si>
+    <t>attribute</t>
+  </si>
+  <si>
+    <t>AuxStoOUT</t>
+  </si>
+  <si>
+    <t>START</t>
+  </si>
+  <si>
+    <t>value</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,6 +217,32 @@
       <family val="2"/>
       <charset val="186"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="186"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="STKFLOW - 14 of 38"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+      <charset val="186"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -199,17 +261,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 10" xfId="1" xr:uid="{81236771-45BA-4F87-83D8-0DEAF9C1680B}"/>
+    <cellStyle name="Normal 3 2" xfId="2" xr:uid="{85AEDC5E-042B-4A26-9E2E-45DB27B8D4A0}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -222,6 +289,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Kristopher Raik" id="{795456CF-7BE3-4FCA-A911-FD9ADA45E4A1}" userId="S::krraik@taltech.ee::b956339b-354b-46f9-8dd3-3584d8dbf762" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -485,39 +558,47 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="C21" dT="2026-01-29T13:24:04.99" personId="{795456CF-7BE3-4FCA-A911-FD9ADA45E4A1}" id="{00A4DA71-5044-48BD-9C8D-CB976CA816BD}">
+    <text>Disabling battery storage related technologies by setting their start time outside the monitored horizon</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:N35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="31.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:14">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:14">
       <c r="E2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:14">
       <c r="I4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:14">
       <c r="B5" s="2" t="s">
         <v>2</v>
       </c>
@@ -558,7 +639,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:14">
       <c r="B6" t="s">
         <v>33</v>
       </c>
@@ -590,7 +671,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:14">
       <c r="B7" t="s">
         <v>37</v>
       </c>
@@ -622,22 +703,22 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:14">
       <c r="B12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:14">
       <c r="B13" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:14">
       <c r="E14" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:14">
       <c r="B15" t="s">
         <v>2</v>
       </c>
@@ -666,7 +747,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:14">
       <c r="B16" t="s">
         <v>34</v>
       </c>
@@ -692,7 +773,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:10">
       <c r="C17" t="s">
         <v>36</v>
       </c>
@@ -709,52 +790,84 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="B22" t="s">
+    <row r="19" spans="2:10">
+      <c r="B19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10">
+      <c r="B20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10">
+      <c r="B21" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21">
+        <v>2100</v>
+      </c>
+      <c r="D21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10">
+      <c r="B28" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" spans="2:10">
+      <c r="B30" t="s">
         <v>21</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D30" t="s">
         <v>25</v>
       </c>
-      <c r="E22">
+      <c r="E30">
         <v>2022</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F30" t="s">
         <v>22</v>
       </c>
-      <c r="G22">
+      <c r="G30">
         <v>1</v>
       </c>
-      <c r="H22">
+      <c r="H30">
         <v>1</v>
       </c>
-      <c r="I22">
+      <c r="I30">
         <v>15</v>
       </c>
-      <c r="J22" t="s">
+      <c r="J30" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
-      <c r="D23" t="s">
+    <row r="31" spans="2:10">
+      <c r="D31" t="s">
         <v>25</v>
       </c>
-      <c r="E23">
+      <c r="E31">
         <v>2050</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F31" t="s">
         <v>22</v>
       </c>
-      <c r="G23">
+      <c r="G31">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:11">
       <c r="B33" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:11">
       <c r="B34" t="s">
         <v>2</v>
       </c>
@@ -786,7 +899,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:11">
       <c r="B35" t="s">
         <v>21</v>
       </c>
@@ -809,5 +922,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
attempt 2: Disabling battery storage related processes by setting their start time outside the horion (2100)
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40442FEC-BF39-4188-88E8-7BB3F5B68F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74120D69-D0C8-4E1A-BFCD-63CF677A0265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="46">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -182,13 +182,16 @@
     <t>attribute</t>
   </si>
   <si>
-    <t>AuxStoOUT</t>
-  </si>
-  <si>
     <t>START</t>
   </si>
   <si>
     <t>value</t>
+  </si>
+  <si>
+    <t>Util Batt Stg</t>
+  </si>
+  <si>
+    <t>EV Batt</t>
   </si>
 </sst>
 </file>
@@ -800,21 +803,29 @@
         <v>41</v>
       </c>
       <c r="C20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D20" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="2:10">
       <c r="B21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C21">
         <v>2100</v>
       </c>
       <c r="D21" t="s">
-        <v>42</v>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10">
+      <c r="C22">
+        <v>2100</v>
+      </c>
+      <c r="D22" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="2:10">

</xml_diff>

<commit_message>
Max wind onshore capacity
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74120D69-D0C8-4E1A-BFCD-63CF677A0265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF4F39C2-63C9-4290-840E-434E02D62E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="enabled" sheetId="1" r:id="rId1"/>
+    <sheet name="disabled" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -54,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="49">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -192,18 +193,35 @@
   </si>
   <si>
     <t>EV Batt</t>
+  </si>
+  <si>
+    <t>~UC_T: 2050</t>
+  </si>
+  <si>
+    <t>Wind onshore</t>
+  </si>
+  <si>
+    <t>UCE_max_wind_onshore_capacity</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="186"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -266,15 +284,16 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -571,7 +590,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:N35"/>
+  <dimension ref="B1:N28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
@@ -668,7 +687,7 @@
         <v>0</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N6" t="s">
         <v>18</v>
@@ -700,7 +719,7 @@
         <v>0</v>
       </c>
       <c r="M7">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N7" t="s">
         <v>38</v>
@@ -828,106 +847,58 @@
         <v>45</v>
       </c>
     </row>
+    <row r="25" spans="2:10">
+      <c r="B25" s="5"/>
+    </row>
+    <row r="26" spans="2:10">
+      <c r="B26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10">
+      <c r="B27" t="s">
+        <v>2</v>
+      </c>
+      <c r="C27" t="s">
+        <v>3</v>
+      </c>
+      <c r="D27" t="s">
+        <v>26</v>
+      </c>
+      <c r="E27" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27" t="s">
+        <v>20</v>
+      </c>
+      <c r="G27">
+        <v>2022</v>
+      </c>
+      <c r="H27">
+        <v>2050</v>
+      </c>
+      <c r="I27" t="s">
+        <v>28</v>
+      </c>
+      <c r="J27" t="s">
+        <v>29</v>
+      </c>
+    </row>
     <row r="28" spans="2:10">
-      <c r="B28" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="30" spans="2:10">
-      <c r="B30" t="s">
-        <v>21</v>
-      </c>
-      <c r="D30" t="s">
-        <v>25</v>
-      </c>
-      <c r="E30">
-        <v>2022</v>
-      </c>
-      <c r="F30" t="s">
-        <v>22</v>
-      </c>
-      <c r="G30">
-        <v>1</v>
-      </c>
-      <c r="H30">
-        <v>1</v>
-      </c>
-      <c r="I30">
-        <v>15</v>
-      </c>
-      <c r="J30" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="31" spans="2:10">
-      <c r="D31" t="s">
-        <v>25</v>
-      </c>
-      <c r="E31">
-        <v>2050</v>
-      </c>
-      <c r="F31" t="s">
-        <v>22</v>
-      </c>
-      <c r="G31">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="2:11">
-      <c r="B33" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="34" spans="2:11">
-      <c r="B34" t="s">
-        <v>2</v>
-      </c>
-      <c r="C34" t="s">
-        <v>24</v>
-      </c>
-      <c r="D34" t="s">
-        <v>26</v>
-      </c>
-      <c r="E34" t="s">
-        <v>27</v>
-      </c>
-      <c r="F34" t="s">
-        <v>20</v>
-      </c>
-      <c r="G34">
-        <v>2022</v>
-      </c>
-      <c r="H34">
-        <v>2050</v>
-      </c>
-      <c r="I34" t="s">
-        <v>28</v>
-      </c>
-      <c r="J34" t="s">
-        <v>29</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="35" spans="2:11">
-      <c r="B35" t="s">
-        <v>21</v>
-      </c>
-      <c r="C35" t="s">
-        <v>25</v>
-      </c>
-      <c r="F35">
-        <v>1</v>
-      </c>
-      <c r="I35">
-        <v>1</v>
-      </c>
-      <c r="J35">
+      <c r="B28" t="s">
+        <v>48</v>
+      </c>
+      <c r="C28" t="s">
+        <v>47</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="I28">
+        <v>1</v>
+      </c>
+      <c r="J28">
         <v>3</v>
-      </c>
-      <c r="K35" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -935,4 +906,116 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{244CCA25-E2DB-463B-BC16-D7A56F0E2E16}">
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3">
+        <v>2022</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>15</v>
+      </c>
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4">
+        <v>2050</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7">
+        <v>2022</v>
+      </c>
+      <c r="G7">
+        <v>2050</v>
+      </c>
+      <c r="H7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" t="s">
+        <v>29</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>3</v>
+      </c>
+      <c r="J8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Commenting out coal and gas utilization
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF4F39C2-63C9-4290-840E-434E02D62E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02CC1C77-7F3F-4BA3-B7CE-FA6A2DA1C5BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="enabled" sheetId="1" r:id="rId1"/>
@@ -601,8 +601,8 @@
     <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:14">

</xml_diff>

<commit_message>
Changing UC_RHSRTS to UC_RHSRT for renewable penetration
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02CC1C77-7F3F-4BA3-B7CE-FA6A2DA1C5BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{387132D9-1594-4E88-B9D1-ECED6F4125AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="47">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -91,12 +91,6 @@
   </si>
   <si>
     <t>EST</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS~0</t>
   </si>
   <si>
     <t>UC_Desc</t>
@@ -208,7 +202,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -256,13 +250,6 @@
     <font>
       <sz val="10"/>
       <name val="STKFLOW - 14 of 38"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-      <charset val="186"/>
     </font>
   </fonts>
   <fills count="2">
@@ -612,7 +599,7 @@
     </row>
     <row r="2" spans="2:14">
       <c r="E2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="2:14">
@@ -652,30 +639,30 @@
         <v>11</v>
       </c>
       <c r="L5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" spans="2:14">
       <c r="B6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H6">
         <v>2035</v>
       </c>
       <c r="I6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -690,24 +677,24 @@
         <v>3</v>
       </c>
       <c r="N6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="2:14">
       <c r="B7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H7">
         <v>2035</v>
       </c>
       <c r="I7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -722,22 +709,22 @@
         <v>3</v>
       </c>
       <c r="N7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="2:14">
       <c r="B12" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="2:14">
       <c r="B13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="2:14">
       <c r="E14" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="2:14">
@@ -748,7 +735,7 @@
         <v>3</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>8</v>
@@ -757,30 +744,30 @@
         <v>9</v>
       </c>
       <c r="G15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
       </c>
       <c r="I15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="2:14">
       <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" t="s">
         <v>34</v>
-      </c>
-      <c r="C16" t="s">
-        <v>36</v>
       </c>
       <c r="E16">
         <v>2030</v>
       </c>
       <c r="F16" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -792,18 +779,18 @@
         <v>5</v>
       </c>
       <c r="J16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="2:10">
       <c r="C17" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E17">
         <v>2035</v>
       </c>
       <c r="F17" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -814,15 +801,15 @@
     </row>
     <row r="19" spans="2:10">
       <c r="B19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="2:10">
       <c r="B20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" t="s">
         <v>41</v>
-      </c>
-      <c r="C20" t="s">
-        <v>43</v>
       </c>
       <c r="D20" t="s">
         <v>3</v>
@@ -830,13 +817,13 @@
     </row>
     <row r="21" spans="2:10">
       <c r="B21" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C21">
         <v>2100</v>
       </c>
       <c r="D21" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="2:10">
@@ -844,7 +831,7 @@
         <v>2100</v>
       </c>
       <c r="D22" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="2:10">
@@ -852,7 +839,7 @@
     </row>
     <row r="26" spans="2:10">
       <c r="B26" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="2:10">
@@ -863,13 +850,13 @@
         <v>3</v>
       </c>
       <c r="D27" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E27" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F27" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G27">
         <v>2022</v>
@@ -878,18 +865,18 @@
         <v>2050</v>
       </c>
       <c r="I27" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="J27" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28" spans="2:10">
       <c r="B28" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C28" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -915,21 +902,21 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D3">
         <v>2022</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -941,18 +928,18 @@
         <v>15</v>
       </c>
       <c r="I3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="C4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D4">
         <v>2050</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -960,7 +947,7 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -968,16 +955,16 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" t="s">
         <v>24</v>
       </c>
-      <c r="C7" t="s">
-        <v>26</v>
-      </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F7">
         <v>2022</v>
@@ -986,21 +973,21 @@
         <v>2050</v>
       </c>
       <c r="H7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="I7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -1012,7 +999,7 @@
         <v>3</v>
       </c>
       <c r="J8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changing renewable penetration constraint logic
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{387132D9-1594-4E88-B9D1-ECED6F4125AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30A2C008-BA49-4DF1-AAB8-3391E56C02E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,14 +55,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="52">
   <si>
     <t>Additions by Kristopher</t>
   </si>
   <si>
-    <t>~UC_T: UC_COMPRD</t>
-  </si>
-  <si>
     <t>UC_N</t>
   </si>
   <si>
@@ -195,7 +192,25 @@
     <t>Wind onshore</t>
   </si>
   <si>
-    <t>UCE_max_wind_onshore_capacity</t>
+    <t>UC_max_wind_onshore_capacity</t>
+  </si>
+  <si>
+    <t>UC_Sets: R_E: AllRegions</t>
+  </si>
+  <si>
+    <t>UC_T: UC_COMPRD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UC_N              </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pset_Set     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PP_RENEW     </t>
+  </si>
+  <si>
+    <t>ELE</t>
   </si>
 </sst>
 </file>
@@ -598,176 +613,213 @@
       </c>
     </row>
     <row r="2" spans="2:14">
-      <c r="E2" t="s">
-        <v>17</v>
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="2:14">
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3">
+        <v>2035</v>
+      </c>
+      <c r="H3">
+        <v>2050</v>
+      </c>
+      <c r="I3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="2:14">
-      <c r="I4" t="s">
-        <v>1</v>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>3</v>
+      </c>
+      <c r="K4" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="2:14">
       <c r="B5" s="2" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="G5" s="2">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2">
         <v>3</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N5" s="2" t="s">
-        <v>12</v>
-      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
     </row>
     <row r="6" spans="2:14">
       <c r="B6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" t="s">
         <v>13</v>
       </c>
-      <c r="G6" t="s">
-        <v>14</v>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>2035</v>
-      </c>
-      <c r="I6" t="s">
-        <v>15</v>
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>1</v>
-      </c>
-      <c r="K6" s="3">
-        <v>-0.75</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
         <v>3</v>
       </c>
-      <c r="N6" t="s">
-        <v>16</v>
+      <c r="K6" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="2:14">
       <c r="B7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" t="s">
         <v>13</v>
       </c>
-      <c r="G7" t="s">
-        <v>14</v>
+      <c r="F7">
+        <v>-0.85</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
       </c>
       <c r="H7">
-        <v>2035</v>
-      </c>
-      <c r="I7" t="s">
-        <v>20</v>
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
       </c>
       <c r="J7">
-        <v>1</v>
-      </c>
-      <c r="K7" s="3">
-        <v>-0.85</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
         <v>3</v>
       </c>
-      <c r="N7" t="s">
-        <v>36</v>
-      </c>
+      <c r="K7" s="3"/>
     </row>
     <row r="12" spans="2:14">
       <c r="B12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="2:14">
       <c r="B13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="2:14">
       <c r="E14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="2:14">
       <c r="B15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
         <v>2</v>
       </c>
-      <c r="C15" t="s">
-        <v>3</v>
-      </c>
       <c r="D15" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" t="s">
         <v>8</v>
       </c>
-      <c r="F15" t="s">
-        <v>9</v>
-      </c>
       <c r="G15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H15" t="s">
+        <v>10</v>
+      </c>
+      <c r="I15" t="s">
+        <v>26</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="I15" t="s">
-        <v>27</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="16" spans="2:14">
       <c r="B16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E16">
         <v>2030</v>
       </c>
       <c r="F16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -779,18 +831,18 @@
         <v>5</v>
       </c>
       <c r="J16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="2:10">
       <c r="C17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E17">
         <v>2035</v>
       </c>
       <c r="F17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G17">
         <v>1</v>
@@ -801,29 +853,29 @@
     </row>
     <row r="19" spans="2:10">
       <c r="B19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" spans="2:10">
       <c r="B20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D20" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="2:10">
       <c r="B21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21">
         <v>2100</v>
       </c>
       <c r="D21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" spans="2:10">
@@ -831,7 +883,7 @@
         <v>2100</v>
       </c>
       <c r="D22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="2:10">
@@ -839,24 +891,24 @@
     </row>
     <row r="26" spans="2:10">
       <c r="B26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="2:10">
       <c r="B27" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
         <v>2</v>
       </c>
-      <c r="C27" t="s">
-        <v>3</v>
-      </c>
       <c r="D27" t="s">
+        <v>23</v>
+      </c>
+      <c r="E27" t="s">
         <v>24</v>
       </c>
-      <c r="E27" t="s">
-        <v>25</v>
-      </c>
       <c r="F27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G27">
         <v>2022</v>
@@ -865,18 +917,18 @@
         <v>2050</v>
       </c>
       <c r="I27" t="s">
+        <v>25</v>
+      </c>
+      <c r="J27" t="s">
         <v>26</v>
-      </c>
-      <c r="J27" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="28" spans="2:10">
       <c r="B28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -897,26 +949,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{244CCA25-E2DB-463B-BC16-D7A56F0E2E16}">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D3">
         <v>2022</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -928,18 +980,18 @@
         <v>15</v>
       </c>
       <c r="I3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="C4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4">
         <v>2050</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -947,24 +999,24 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" t="s">
         <v>24</v>
       </c>
-      <c r="D7" t="s">
-        <v>25</v>
-      </c>
       <c r="E7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7">
         <v>2022</v>
@@ -973,21 +1025,21 @@
         <v>2050</v>
       </c>
       <c r="H7" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" t="s">
         <v>26</v>
       </c>
-      <c r="I7" t="s">
-        <v>27</v>
-      </c>
       <c r="J7" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -999,7 +1051,122 @@
         <v>3</v>
       </c>
       <c r="J8" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="D14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="H16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
+      <c r="A17" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
+      <c r="A18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18">
+        <v>2035</v>
+      </c>
+      <c r="H18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I18">
+        <v>1</v>
+      </c>
+      <c r="J18" s="3">
+        <v>-0.75</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>3</v>
+      </c>
+      <c r="M18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19">
+        <v>2035</v>
+      </c>
+      <c r="H19" t="s">
+        <v>19</v>
+      </c>
+      <c r="I19">
+        <v>1</v>
+      </c>
+      <c r="J19" s="3">
+        <v>-0.85</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>3</v>
+      </c>
+      <c r="M19" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changing renewable penetration constraint logic part 2
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30A2C008-BA49-4DF1-AAB8-3391E56C02E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24114868-C520-450D-8CE9-548825697EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="enabled" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="50">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -201,16 +201,10 @@
     <t>UC_T: UC_COMPRD</t>
   </si>
   <si>
-    <t xml:space="preserve">UC_N              </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pset_Set     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PP_RENEW     </t>
-  </si>
-  <si>
     <t>ELE</t>
+  </si>
+  <si>
+    <t>-PP_RENEW</t>
   </si>
 </sst>
 </file>
@@ -289,13 +283,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -592,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:N28"/>
+  <dimension ref="B1:N34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
@@ -612,156 +607,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="2:14">
-      <c r="B2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="2:14">
-      <c r="B3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3">
-        <v>2035</v>
-      </c>
-      <c r="H3">
-        <v>2050</v>
-      </c>
-      <c r="I3" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="2:14">
-      <c r="B4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>3</v>
-      </c>
-      <c r="K4" t="s">
-        <v>15</v>
-      </c>
-    </row>
     <row r="5" spans="2:14">
-      <c r="B5" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="2">
-        <v>0.75</v>
-      </c>
-      <c r="G5" s="2">
-        <v>1</v>
-      </c>
-      <c r="H5" s="2">
-        <v>1</v>
-      </c>
-      <c r="I5" s="2">
-        <v>0</v>
-      </c>
-      <c r="J5" s="2">
-        <v>3</v>
-      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
     </row>
     <row r="6" spans="2:14">
-      <c r="B6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>3</v>
-      </c>
-      <c r="K6" t="s">
-        <v>35</v>
-      </c>
+      <c r="K6" s="3"/>
     </row>
     <row r="7" spans="2:14">
-      <c r="B7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" t="s">
-        <v>51</v>
-      </c>
-      <c r="D7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7">
-        <v>-0.85</v>
-      </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7">
-        <v>0</v>
-      </c>
-      <c r="J7">
-        <v>3</v>
-      </c>
       <c r="K7" s="3"/>
     </row>
     <row r="12" spans="2:14">
@@ -834,7 +698,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="2:10">
+    <row r="17" spans="2:11">
       <c r="C17" t="s">
         <v>33</v>
       </c>
@@ -851,12 +715,12 @@
         <v>2.1</v>
       </c>
     </row>
-    <row r="19" spans="2:10">
+    <row r="19" spans="2:11">
       <c r="B19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="2:10">
+    <row r="20" spans="2:11">
       <c r="B20" t="s">
         <v>38</v>
       </c>
@@ -867,7 +731,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:10">
+    <row r="21" spans="2:11">
       <c r="B21" t="s">
         <v>39</v>
       </c>
@@ -878,7 +742,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="2:10">
+    <row r="22" spans="2:11">
       <c r="C22">
         <v>2100</v>
       </c>
@@ -886,15 +750,15 @@
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="2:10">
+    <row r="25" spans="2:11">
       <c r="B25" s="5"/>
     </row>
-    <row r="26" spans="2:10">
+    <row r="26" spans="2:11">
       <c r="B26" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="27" spans="2:10">
+    <row r="27" spans="2:11">
       <c r="B27" t="s">
         <v>1</v>
       </c>
@@ -923,7 +787,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="2:10">
+    <row r="28" spans="2:11">
       <c r="B28" t="s">
         <v>45</v>
       </c>
@@ -938,6 +802,95 @@
       </c>
       <c r="J28">
         <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11">
+      <c r="B31" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="2:11">
+      <c r="B32" t="s">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2</v>
+      </c>
+      <c r="D32" t="s">
+        <v>6</v>
+      </c>
+      <c r="E32" t="s">
+        <v>24</v>
+      </c>
+      <c r="F32" t="s">
+        <v>8</v>
+      </c>
+      <c r="G32" t="s">
+        <v>9</v>
+      </c>
+      <c r="H32">
+        <v>2035</v>
+      </c>
+      <c r="I32">
+        <v>2050</v>
+      </c>
+      <c r="J32" t="s">
+        <v>25</v>
+      </c>
+      <c r="K32" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11">
+      <c r="B33" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" t="s">
+        <v>48</v>
+      </c>
+      <c r="F33" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33">
+        <v>0.75</v>
+      </c>
+      <c r="H33">
+        <v>1</v>
+      </c>
+      <c r="I33">
+        <v>1</v>
+      </c>
+      <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11">
+      <c r="C34" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D34" t="s">
+        <v>48</v>
+      </c>
+      <c r="F34" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34">
+        <v>-0.35</v>
+      </c>
+      <c r="H34">
+        <v>1</v>
+      </c>
+      <c r="I34">
+        <v>1</v>
+      </c>
+      <c r="J34">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changing renewable penetration constraint logic part 3
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24114868-C520-450D-8CE9-548825697EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D4A1EAC-4231-40DA-B17B-AE7C7EC48845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="enabled" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="49">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -199,9 +199,6 @@
   </si>
   <si>
     <t>UC_T: UC_COMPRD</t>
-  </si>
-  <si>
-    <t>ELE</t>
   </si>
   <si>
     <t>-PP_RENEW</t>
@@ -849,7 +846,7 @@
         <v>12</v>
       </c>
       <c r="D33" t="s">
-        <v>48</v>
+        <v>13</v>
       </c>
       <c r="F33" t="s">
         <v>14</v>
@@ -872,10 +869,10 @@
     </row>
     <row r="34" spans="2:11">
       <c r="C34" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D34" t="s">
-        <v>48</v>
+        <v>13</v>
       </c>
       <c r="F34" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
Changing renewable penetration constraint logic part 4
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D4A1EAC-4231-40DA-B17B-AE7C7EC48845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24189282-9371-4DC3-9859-004E86789836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -852,7 +852,7 @@
         <v>14</v>
       </c>
       <c r="G33">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="H33">
         <v>1</v>

</xml_diff>

<commit_message>
Changing renewable penetration constraint logic part 5
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24189282-9371-4DC3-9859-004E86789836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85E6676C-9DF0-44F0-ADCD-BB5B72A64A19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="enabled" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="49">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -1062,9 +1062,6 @@
       <c r="B18" t="s">
         <v>12</v>
       </c>
-      <c r="F18" t="s">
-        <v>13</v>
-      </c>
       <c r="G18">
         <v>2035</v>
       </c>
@@ -1093,9 +1090,6 @@
       </c>
       <c r="B19" t="s">
         <v>12</v>
-      </c>
-      <c r="F19" t="s">
-        <v>13</v>
       </c>
       <c r="G19">
         <v>2035</v>

</xml_diff>

<commit_message>
Adding batteries to 2030
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967C8855-9A41-44C2-89E4-BE626AA94222}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEF068C8-F0AF-43CA-80C5-0936D6C8D4C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -743,7 +743,7 @@
         <v>39</v>
       </c>
       <c r="C21">
-        <v>2100</v>
+        <v>2030</v>
       </c>
       <c r="D21" t="s">
         <v>41</v>
@@ -751,7 +751,7 @@
     </row>
     <row r="22" spans="2:11">
       <c r="C22">
-        <v>2100</v>
+        <v>2030</v>
       </c>
       <c r="D22" t="s">
         <v>42</v>

</xml_diff>

<commit_message>
Updating oil shale constraint
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F8A969-709E-4F88-9CC0-9FE4DBEA77DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4EE5F22-3274-46E4-AEAE-20D356154488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="enabled" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
     <author>tc={00A4DA71-5044-48BD-9C8D-CB976CA816BD}</author>
   </authors>
   <commentList>
-    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{00A4DA71-5044-48BD-9C8D-CB976CA816BD}">
+    <comment ref="C24" authorId="0" shapeId="0" xr:uid="{00A4DA71-5044-48BD-9C8D-CB976CA816BD}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="53">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -211,6 +211,9 @@
   </si>
   <si>
     <t>COAL</t>
+  </si>
+  <si>
+    <t>UC_T:UC_RHSRT</t>
   </si>
 </sst>
 </file>
@@ -586,7 +589,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C21" dT="2026-01-29T13:24:04.99" personId="{795456CF-7BE3-4FCA-A911-FD9ADA45E4A1}" id="{00A4DA71-5044-48BD-9C8D-CB976CA816BD}">
+  <threadedComment ref="C24" dT="2026-01-29T13:24:04.99" personId="{795456CF-7BE3-4FCA-A911-FD9ADA45E4A1}" id="{00A4DA71-5044-48BD-9C8D-CB976CA816BD}">
     <text>Disabling battery storage related technologies by setting their start time outside the monitored horizon</text>
   </threadedComment>
 </ThreadedComments>
@@ -594,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:N32"/>
+  <dimension ref="B1:N31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
@@ -722,156 +725,139 @@
         <v>2.1</v>
       </c>
     </row>
+    <row r="18" spans="2:11">
+      <c r="B18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18">
+        <v>2030</v>
+      </c>
+      <c r="F18" t="s">
+        <v>19</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>0.28299999999999997</v>
+      </c>
+      <c r="I18">
+        <v>5</v>
+      </c>
+    </row>
     <row r="19" spans="2:11">
-      <c r="B19" t="s">
+      <c r="D19" t="s">
+        <v>51</v>
+      </c>
+      <c r="E19">
+        <v>2050</v>
+      </c>
+      <c r="F19" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="2:11">
+      <c r="B22" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="2:11">
-      <c r="B20" t="s">
+    <row r="23" spans="2:11">
+      <c r="B23" t="s">
         <v>38</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C23" t="s">
         <v>40</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D23" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:11">
-      <c r="B21" t="s">
+    <row r="24" spans="2:11">
+      <c r="B24" t="s">
         <v>39</v>
       </c>
-      <c r="C21">
+      <c r="C24">
         <v>2030</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D24" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="2:11">
-      <c r="C22">
+    <row r="25" spans="2:11">
+      <c r="C25">
         <v>2030</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D25" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="2:11">
-      <c r="B25" s="5"/>
-    </row>
-    <row r="26" spans="2:11">
-      <c r="B26" t="s">
+    <row r="28" spans="2:11">
+      <c r="B28" s="5"/>
+    </row>
+    <row r="29" spans="2:11">
+      <c r="B29" t="s">
         <v>43</v>
-      </c>
-    </row>
-    <row r="27" spans="2:11">
-      <c r="B27" t="s">
-        <v>1</v>
-      </c>
-      <c r="C27" t="s">
-        <v>2</v>
-      </c>
-      <c r="D27" t="s">
-        <v>21</v>
-      </c>
-      <c r="E27" t="s">
-        <v>23</v>
-      </c>
-      <c r="F27" t="s">
-        <v>24</v>
-      </c>
-      <c r="G27" t="s">
-        <v>17</v>
-      </c>
-      <c r="H27">
-        <v>2022</v>
-      </c>
-      <c r="I27">
-        <v>2050</v>
-      </c>
-      <c r="J27" t="s">
-        <v>25</v>
-      </c>
-      <c r="K27" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="2:11">
-      <c r="B28" t="s">
-        <v>45</v>
-      </c>
-      <c r="C28" t="s">
-        <v>44</v>
-      </c>
-      <c r="G28">
-        <v>1</v>
-      </c>
-      <c r="J28">
-        <v>1</v>
-      </c>
-      <c r="K28">
-        <v>3</v>
       </c>
     </row>
     <row r="30" spans="2:11">
       <c r="B30" t="s">
-        <v>29</v>
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
+        <v>2</v>
+      </c>
+      <c r="D30" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" t="s">
+        <v>23</v>
+      </c>
+      <c r="F30" t="s">
+        <v>24</v>
+      </c>
+      <c r="G30" t="s">
+        <v>17</v>
+      </c>
+      <c r="H30">
+        <v>2022</v>
+      </c>
+      <c r="I30">
+        <v>2050</v>
+      </c>
+      <c r="J30" t="s">
+        <v>25</v>
+      </c>
+      <c r="K30" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="31" spans="2:11">
       <c r="B31" t="s">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="C31" t="s">
-        <v>2</v>
-      </c>
-      <c r="D31" t="s">
-        <v>21</v>
-      </c>
-      <c r="E31" t="s">
-        <v>23</v>
-      </c>
-      <c r="F31" t="s">
-        <v>8</v>
-      </c>
-      <c r="G31" t="s">
-        <v>24</v>
-      </c>
-      <c r="H31" t="s">
-        <v>17</v>
-      </c>
-      <c r="I31">
-        <v>2030</v>
+        <v>44</v>
+      </c>
+      <c r="G31">
+        <v>1</v>
       </c>
       <c r="J31">
-        <v>2050</v>
-      </c>
-      <c r="K31" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="32" spans="2:11">
-      <c r="B32" t="s">
-        <v>50</v>
-      </c>
-      <c r="D32" t="s">
-        <v>51</v>
-      </c>
-      <c r="F32" t="s">
-        <v>19</v>
-      </c>
-      <c r="H32">
-        <v>1</v>
-      </c>
-      <c r="I32">
-        <v>0.28299999999999997</v>
-      </c>
-      <c r="J32">
-        <v>0</v>
-      </c>
-      <c r="K32">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="K31">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -883,7 +869,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{244CCA25-E2DB-463B-BC16-D7A56F0E2E16}">
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1166,6 +1152,66 @@
     <row r="25" spans="1:13">
       <c r="B25" s="7"/>
     </row>
+    <row r="29" spans="1:13">
+      <c r="E29" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
+      <c r="A30" t="s">
+        <v>1</v>
+      </c>
+      <c r="B30" t="s">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>21</v>
+      </c>
+      <c r="D30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E30" t="s">
+        <v>8</v>
+      </c>
+      <c r="F30" t="s">
+        <v>24</v>
+      </c>
+      <c r="G30" t="s">
+        <v>17</v>
+      </c>
+      <c r="H30">
+        <v>2030</v>
+      </c>
+      <c r="I30">
+        <v>2050</v>
+      </c>
+      <c r="J30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
+      <c r="A31" t="s">
+        <v>50</v>
+      </c>
+      <c r="C31" t="s">
+        <v>51</v>
+      </c>
+      <c r="E31" t="s">
+        <v>19</v>
+      </c>
+      <c r="G31">
+        <v>1</v>
+      </c>
+      <c r="H31">
+        <v>0.28299999999999997</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updating oil shale constraint attempt 2
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4EE5F22-3274-46E4-AEAE-20D356154488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97C9408E-D695-46D3-8687-F7380F6B59CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="54">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -214,6 +214,9 @@
   </si>
   <si>
     <t>UC_T:UC_RHSRT</t>
+  </si>
+  <si>
+    <t>Subcritical Coal,Supercritical Coal</t>
   </si>
 </sst>
 </file>
@@ -601,7 +604,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -702,7 +705,7 @@
         <v>2</v>
       </c>
       <c r="I16">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J16" t="s">
         <v>32</v>
@@ -729,8 +732,8 @@
       <c r="B18" t="s">
         <v>50</v>
       </c>
-      <c r="D18" t="s">
-        <v>51</v>
+      <c r="C18" t="s">
+        <v>53</v>
       </c>
       <c r="E18">
         <v>2030</v>
@@ -745,12 +748,12 @@
         <v>0.28299999999999997</v>
       </c>
       <c r="I18">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="2:11">
-      <c r="D19" t="s">
-        <v>51</v>
+      <c r="C19" t="s">
+        <v>53</v>
       </c>
       <c r="E19">
         <v>2050</v>
@@ -763,9 +766,6 @@
       </c>
       <c r="H19">
         <v>0</v>
-      </c>
-      <c r="I19">
-        <v>5</v>
       </c>
     </row>
     <row r="22" spans="2:11">

</xml_diff>

<commit_message>
Updating oil shale constraint attempt 3
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97C9408E-D695-46D3-8687-F7380F6B59CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DFB47D-8AAC-48FA-B45B-03FF7387AD6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -736,7 +736,7 @@
         <v>53</v>
       </c>
       <c r="E18">
-        <v>2030</v>
+        <v>2025</v>
       </c>
       <c r="F18" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Updating oil shale constraint attempt 4
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_ENMAK.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DFB47D-8AAC-48FA-B45B-03FF7387AD6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E32DB92-7F66-44E0-8FDD-78192383FB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="enabled" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
     <author>tc={00A4DA71-5044-48BD-9C8D-CB976CA816BD}</author>
   </authors>
   <commentList>
-    <comment ref="C24" authorId="0" shapeId="0" xr:uid="{00A4DA71-5044-48BD-9C8D-CB976CA816BD}">
+    <comment ref="C26" authorId="0" shapeId="0" xr:uid="{00A4DA71-5044-48BD-9C8D-CB976CA816BD}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="53">
   <si>
     <t>Additions by Kristopher</t>
   </si>
@@ -139,9 +139,6 @@
   </si>
   <si>
     <t>*UC_T: 2050</t>
-  </si>
-  <si>
-    <t>~UC_Sets: T_E:</t>
   </si>
   <si>
     <t>~UC_T:UC_RHSRT</t>
@@ -295,7 +292,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -303,7 +300,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -592,7 +588,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C24" dT="2026-01-29T13:24:04.99" personId="{795456CF-7BE3-4FCA-A911-FD9ADA45E4A1}" id="{00A4DA71-5044-48BD-9C8D-CB976CA816BD}">
+  <threadedComment ref="C26" dT="2026-01-29T13:24:04.99" personId="{795456CF-7BE3-4FCA-A911-FD9ADA45E4A1}" id="{00A4DA71-5044-48BD-9C8D-CB976CA816BD}">
     <text>Disabling battery storage related technologies by setting their start time outside the monitored horizon</text>
   </threadedComment>
 </ThreadedComments>
@@ -600,7 +596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:N31"/>
+  <dimension ref="B1:N33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="31.85546875" bestFit="1" customWidth="1"/>
@@ -646,14 +642,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="13" spans="2:14">
-      <c r="B13" t="s">
-        <v>28</v>
-      </c>
-    </row>
     <row r="14" spans="2:14">
       <c r="E14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="2:14">
@@ -687,10 +678,10 @@
     </row>
     <row r="16" spans="2:14">
       <c r="B16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E16">
         <v>2030</v>
@@ -704,16 +695,13 @@
       <c r="H16">
         <v>2</v>
       </c>
-      <c r="I16">
-        <v>3</v>
-      </c>
       <c r="J16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="2:11">
       <c r="C17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E17">
         <v>2035</v>
@@ -729,34 +717,28 @@
       </c>
     </row>
     <row r="18" spans="2:11">
-      <c r="B18" t="s">
-        <v>50</v>
-      </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="E18">
-        <v>2025</v>
+        <v>0</v>
       </c>
       <c r="F18" t="s">
-        <v>19</v>
-      </c>
-      <c r="G18">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="H18">
-        <v>0.28299999999999997</v>
-      </c>
-      <c r="I18">
         <v>3</v>
       </c>
     </row>
     <row r="19" spans="2:11">
+      <c r="B19" t="s">
+        <v>49</v>
+      </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E19">
-        <v>2050</v>
+        <v>2030</v>
       </c>
       <c r="F19" t="s">
         <v>19</v>
@@ -765,98 +747,129 @@
         <v>1</v>
       </c>
       <c r="H19">
+        <v>0.28299999999999997</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11">
+      <c r="C20" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20">
+        <v>2050</v>
+      </c>
+      <c r="F20" t="s">
+        <v>19</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:11">
-      <c r="B22" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" spans="2:11">
-      <c r="B23" t="s">
-        <v>38</v>
-      </c>
-      <c r="C23" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" t="s">
-        <v>2</v>
+    <row r="21" spans="2:11">
+      <c r="C21" t="s">
+        <v>52</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21" t="s">
+        <v>19</v>
+      </c>
+      <c r="H21">
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="2:11">
       <c r="B24" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11">
+      <c r="B25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" t="s">
         <v>39</v>
       </c>
-      <c r="C24">
+      <c r="D25" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11">
+      <c r="B26" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26">
         <v>2030</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11">
+      <c r="C27">
+        <v>2030</v>
+      </c>
+      <c r="D27" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="25" spans="2:11">
-      <c r="C25">
-        <v>2030</v>
-      </c>
-      <c r="D25" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="28" spans="2:11">
-      <c r="B28" s="5"/>
-    </row>
-    <row r="29" spans="2:11">
-      <c r="B29" t="s">
-        <v>43</v>
-      </c>
-    </row>
     <row r="30" spans="2:11">
-      <c r="B30" t="s">
-        <v>1</v>
-      </c>
-      <c r="C30" t="s">
-        <v>2</v>
-      </c>
-      <c r="D30" t="s">
-        <v>21</v>
-      </c>
-      <c r="E30" t="s">
-        <v>23</v>
-      </c>
-      <c r="F30" t="s">
-        <v>24</v>
-      </c>
-      <c r="G30" t="s">
-        <v>17</v>
-      </c>
-      <c r="H30">
-        <v>2022</v>
-      </c>
-      <c r="I30">
-        <v>2050</v>
-      </c>
-      <c r="J30" t="s">
-        <v>25</v>
-      </c>
-      <c r="K30" t="s">
-        <v>26</v>
-      </c>
+      <c r="B30" s="5"/>
     </row>
     <row r="31" spans="2:11">
       <c r="B31" t="s">
-        <v>45</v>
-      </c>
-      <c r="C31" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="32" spans="2:11">
+      <c r="B32" t="s">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2</v>
+      </c>
+      <c r="D32" t="s">
+        <v>21</v>
+      </c>
+      <c r="E32" t="s">
+        <v>23</v>
+      </c>
+      <c r="F32" t="s">
+        <v>24</v>
+      </c>
+      <c r="G32" t="s">
+        <v>17</v>
+      </c>
+      <c r="H32">
+        <v>2022</v>
+      </c>
+      <c r="I32">
+        <v>2050</v>
+      </c>
+      <c r="J32" t="s">
+        <v>25</v>
+      </c>
+      <c r="K32" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="2:11">
+      <c r="B33" t="s">
         <v>44</v>
       </c>
-      <c r="G31">
-        <v>1</v>
-      </c>
-      <c r="J31">
-        <v>1</v>
-      </c>
-      <c r="K31">
+      <c r="C33" t="s">
+        <v>43</v>
+      </c>
+      <c r="G33">
+        <v>1</v>
+      </c>
+      <c r="J33">
+        <v>1</v>
+      </c>
+      <c r="K33">
         <v>3</v>
       </c>
     </row>
@@ -874,7 +887,7 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -976,12 +989,12 @@
     </row>
     <row r="14" spans="1:10">
       <c r="D14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="H16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -1027,7 +1040,7 @@
     </row>
     <row r="18" spans="1:13">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18" t="s">
         <v>12</v>
@@ -1059,7 +1072,7 @@
     </row>
     <row r="19" spans="1:13">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B19" t="s">
         <v>12</v>
@@ -1086,12 +1099,12 @@
         <v>3</v>
       </c>
       <c r="M19" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:13">
       <c r="A22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -1128,10 +1141,10 @@
     </row>
     <row r="24" spans="1:13">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C24" t="s">
         <v>13</v>
@@ -1150,11 +1163,11 @@
       </c>
     </row>
     <row r="25" spans="1:13">
-      <c r="B25" s="7"/>
+      <c r="B25" s="6"/>
     </row>
     <row r="29" spans="1:13">
       <c r="E29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -1191,10 +1204,10 @@
     </row>
     <row r="31" spans="1:13">
       <c r="A31" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" t="s">
         <v>50</v>
-      </c>
-      <c r="C31" t="s">
-        <v>51</v>
       </c>
       <c r="E31" t="s">
         <v>19</v>

</xml_diff>